<commit_message>
Correção da ULA. Troca da implementação comportamental por portas lógicas
</commit_message>
<xml_diff>
--- a/ALU/ULA.xlsx
+++ b/ALU/ULA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SD\ALU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C17916C8-5FEE-4CFA-B67D-40136D652C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6F6A270-D767-4580-BF00-052EDA78F182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E28DD45A-EB33-46FC-9D3E-1B6B3BFB29DF}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
   <si>
     <t>x</t>
   </si>
@@ -78,6 +78,21 @@
   </si>
   <si>
     <t>b'</t>
+  </si>
+  <si>
+    <t>x'y'z+x'yz'</t>
+  </si>
+  <si>
+    <t>x'(y xor z)</t>
+  </si>
+  <si>
+    <t>x'y'(zb'+z'b)</t>
+  </si>
+  <si>
+    <t>x'y'(z xor b)</t>
+  </si>
+  <si>
+    <t>x'a+xy'z'ab+xy'z(a+b)+xyz'(a xor b)+xyza'</t>
   </si>
 </sst>
 </file>
@@ -101,24 +116,36 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.499984740745262"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -127,10 +154,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,186 +496,210 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0168F4-C50F-47DA-9556-AB6B188E2B3D}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="H1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6">
+        <v>0</v>
+      </c>
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>0</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2">
-        <v>1</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="H2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1">
+        <v>0</v>
+      </c>
+      <c r="C3" s="6">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>0</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4" s="2">
-        <v>1</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="H3" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>0</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>0</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="F4" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>0</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>1</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0</v>
-      </c>
-      <c r="E6" s="2" t="s">
+      <c r="F5" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>1</v>
+      </c>
+      <c r="B6" s="1">
+        <v>0</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="F6" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>1</v>
+      </c>
+      <c r="B7" s="1">
+        <v>0</v>
+      </c>
+      <c r="C7" s="6">
+        <v>1</v>
+      </c>
+      <c r="D7" s="5">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>1</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0</v>
-      </c>
-      <c r="E8" s="2" t="s">
+      <c r="F7" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>1</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>1</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9" s="2">
-        <v>0</v>
-      </c>
-      <c r="E9" s="2" t="s">
+      <c r="F8" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>1</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1</v>
+      </c>
+      <c r="C9" s="6">
+        <v>1</v>
+      </c>
+      <c r="D9" s="5">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>